<commit_message>
ISSUE-CELLSCLOUD-14165: Enhancement of Aspose.Cells Cloud SDK with AI/ML capabilities.
</commit_message>
<xml_diff>
--- a/testdata/Home inventory.xlsx
+++ b/testdata/Home inventory.xlsx
@@ -1,22 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cells.cloud-sdk-net\testdata\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28817"/>
+  <workbookPr filterPrivacy="1" showInkAnnotation="0"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB3D1B26-1107-4FC6-B035-BD49DBC37F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="23145" windowHeight="8955"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Home Contents Inventory List" sheetId="1" r:id="rId1"/>
     <sheet name="Room Lookup" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="Slicer_Room__area">#N/A</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Home Contents Inventory List'!$B$1:$L$9</definedName>
     <definedName name="ColumnTitle1">Inventory[[#Headers],[Item '#]]</definedName>
     <definedName name="ColumnTitle2">RoomLookup[[#Headers],[Room/Area]]</definedName>
@@ -27,9 +22,13 @@
     <definedName name="RowTitleRegion2..I2">'Home Contents Inventory List'!$G$2</definedName>
     <definedName name="RowTitleRegion3..D8">'Home Contents Inventory List'!$C$3</definedName>
     <definedName name="RowTitleRegion4..I8">'Home Contents Inventory List'!$H$3</definedName>
+    <definedName name="Slicer_Room__area">#N/A</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr/>
+    </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{46BE6895-7355-4a93-B00E-2C351335B9C9}">
       <x15:slicerCaches xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
         <x14:slicerCache r:id="rId3"/>
@@ -53,242 +52,313 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="72">
   <si>
-    <t xml:space="preserve">  </t>
-  </si>
-  <si>
-    <t>Home Inventory</t>
-  </si>
-  <si>
-    <t>Contents List</t>
-  </si>
-  <si>
-    <t>House icon is in this cell</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> TOTAL ESTIMATED VALUE OF ALL ITEMS:</t>
-  </si>
-  <si>
-    <t>INVENTORY DATE:</t>
-  </si>
-  <si>
-    <t>Person icon is in this cell</t>
-  </si>
-  <si>
-    <t>NAME:</t>
-  </si>
-  <si>
-    <t>Roy Wang</t>
-  </si>
-  <si>
-    <t>Insurance company:</t>
-  </si>
-  <si>
-    <t>Ping An Insurance Company</t>
-  </si>
-  <si>
-    <t>Insurance company phone:</t>
-  </si>
-  <si>
-    <t>Envelope is in this cell</t>
-  </si>
-  <si>
-    <t>ADDRESS:</t>
-  </si>
-  <si>
-    <t>China Nanjing</t>
-  </si>
-  <si>
-    <t>Insurance company policy number:</t>
-  </si>
-  <si>
-    <t>Insurance agent:</t>
-  </si>
-  <si>
-    <t>Agent of Ping An Insurance Company in Nanjing</t>
-  </si>
-  <si>
-    <t>Phone icon is in this cell</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>roy.wang@aspose.com</t>
-  </si>
-  <si>
-    <t>Insurance agent phone:</t>
-  </si>
-  <si>
-    <t>Insurance agent address:</t>
-  </si>
-  <si>
-    <t>Ping'an Road, Gulou District, Nanjing China</t>
-  </si>
-  <si>
-    <t>A slicer is in cells B9 through J9. To filter inventory list, select a room from the slicer in this cell. Press and hold CTRL to select multiple rooms.</t>
-  </si>
-  <si>
-    <t>Item #</t>
-  </si>
-  <si>
-    <t>Room/area</t>
-  </si>
-  <si>
-    <t>Item/description</t>
-  </si>
-  <si>
-    <t>Make/model</t>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Photo?</t>
   </si>
   <si>
     <t>Serial number/
 ID number</t>
   </si>
   <si>
+    <t>Where purchased</t>
+  </si>
+  <si>
+    <t>Purchase
+ price</t>
+  </si>
+  <si>
+    <t>Living Room</t>
+  </si>
+  <si>
+    <t>Dining Room</t>
+  </si>
+  <si>
+    <t>Kitchen</t>
+  </si>
+  <si>
+    <t>Master Bedroom</t>
+  </si>
+  <si>
+    <t>Bedroom 1</t>
+  </si>
+  <si>
+    <t>Bedroom 2</t>
+  </si>
+  <si>
+    <t>Bedroom 3</t>
+  </si>
+  <si>
+    <t>Garage</t>
+  </si>
+  <si>
+    <t>Family Room</t>
+  </si>
+  <si>
+    <t>Home Office</t>
+  </si>
+  <si>
+    <t>Room/Area</t>
+  </si>
+  <si>
+    <t>Online</t>
+  </si>
+  <si>
+    <t>33XCBH3</t>
+  </si>
+  <si>
+    <t>55-678B</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Item 1</t>
+  </si>
+  <si>
+    <t>Item 2</t>
+  </si>
+  <si>
+    <t>Insurance agent:</t>
+  </si>
+  <si>
+    <t>Insurance agent phone:</t>
+  </si>
+  <si>
+    <t>Insurance company:</t>
+  </si>
+  <si>
+    <t>Insurance company phone:</t>
+  </si>
+  <si>
+    <t>Insurance company policy number:</t>
+  </si>
+  <si>
     <t>Date
 purchased</t>
   </si>
   <si>
-    <t>Where purchased</t>
-  </si>
-  <si>
-    <t>Purchase
- price</t>
-  </si>
-  <si>
     <t>Estimated
 current value</t>
   </si>
   <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Photo?</t>
-  </si>
-  <si>
-    <t>Living Room</t>
-  </si>
-  <si>
-    <t>Item 1</t>
+    <t>TOTALS</t>
+  </si>
+  <si>
+    <t>Computer Store</t>
+  </si>
+  <si>
+    <t>Item #</t>
+  </si>
+  <si>
+    <t>Insurance agent address:</t>
+  </si>
+  <si>
+    <t>NAME:</t>
+  </si>
+  <si>
+    <t>ADDRESS:</t>
+  </si>
+  <si>
+    <t>Basement</t>
+  </si>
+  <si>
+    <t>Item 3</t>
+  </si>
+  <si>
+    <t>7865SS-J3</t>
+  </si>
+  <si>
+    <t>Furniture store</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TOTAL ESTIMATED VALUE OF ALL ITEMS:</t>
+  </si>
+  <si>
+    <t>INVENTORY DATE:</t>
+  </si>
+  <si>
+    <t>Item 4</t>
+  </si>
+  <si>
+    <t>768087</t>
+  </si>
+  <si>
+    <t>Item 5</t>
+  </si>
+  <si>
+    <t>80-JBNR</t>
+  </si>
+  <si>
+    <t>Bedroom 4</t>
   </si>
   <si>
     <t>Manufacturer 1</t>
   </si>
   <si>
-    <t>33XCBH3</t>
-  </si>
-  <si>
-    <t>Online</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Home Office</t>
-  </si>
-  <si>
-    <t>Item 2</t>
-  </si>
-  <si>
     <t>Manufacturer 2</t>
   </si>
   <si>
-    <t>55-678B</t>
-  </si>
-  <si>
-    <t>Computer Store</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Item 3</t>
-  </si>
-  <si>
     <t>Manufacturer 3</t>
   </si>
   <si>
-    <t>7865SS-J3</t>
-  </si>
-  <si>
-    <t>Furniture store</t>
-  </si>
-  <si>
-    <t>Dining Room</t>
-  </si>
-  <si>
-    <t>Item 4</t>
-  </si>
-  <si>
     <t>Manufacturer 4</t>
   </si>
   <si>
-    <t>768087</t>
-  </si>
-  <si>
-    <t>Family Room</t>
-  </si>
-  <si>
-    <t>Item 5</t>
-  </si>
-  <si>
     <t>Manufacturer 5</t>
   </si>
   <si>
-    <t>80-JBNR</t>
-  </si>
-  <si>
-    <t>TOTALS</t>
+    <t>Home Inventory</t>
+  </si>
+  <si>
+    <t>Contents List</t>
+  </si>
+  <si>
+    <t>Modify or add entries to this list. Simply type over an existing entry or add a new entry directly below the last row of the table.</t>
+  </si>
+  <si>
+    <t>House icon is in this cell</t>
+  </si>
+  <si>
+    <t>Room/area</t>
+  </si>
+  <si>
+    <t>Item/description</t>
+  </si>
+  <si>
+    <t>Make/model</t>
   </si>
   <si>
     <t>Room Lookup</t>
   </si>
   <si>
-    <t>Modify or add entries to this list. Simply type over an existing entry or add a new entry directly below the last row of the table.</t>
-  </si>
-  <si>
-    <t>Room/Area</t>
-  </si>
-  <si>
-    <t>Basement</t>
-  </si>
-  <si>
-    <t>Bedroom 1</t>
-  </si>
-  <si>
-    <t>Bedroom 2</t>
-  </si>
-  <si>
-    <t>Bedroom 3</t>
-  </si>
-  <si>
-    <t>Bedroom 4</t>
-  </si>
-  <si>
-    <t>Garage</t>
-  </si>
-  <si>
-    <t>Kitchen</t>
-  </si>
-  <si>
-    <t>Master Bedroom</t>
+    <t>Person icon is in this cell</t>
+  </si>
+  <si>
+    <t>Envelope is in this cell</t>
+  </si>
+  <si>
+    <t>Phone icon is in this cell</t>
+  </si>
+  <si>
+    <t>A slicer is in cells B9 through J9. To filter inventory list, select a room from the slicer in this cell. Press and hold CTRL to select multiple rooms.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t>Roy Wang</t>
+  </si>
+  <si>
+    <t>China Nanjing</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>roy.wang@aspose.com</t>
+  </si>
+  <si>
+    <t>Ping An Insurance Company</t>
+  </si>
+  <si>
+    <t>Agent of Ping An Insurance Company in Nanjing</t>
+  </si>
+  <si>
+    <t>Ping'an Road, Gulou District, Nanjing China</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <numFmts count="3">
     <numFmt numFmtId="7" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="176" formatCode="0_);\(0\)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="[&lt;=9999999]###\-####;\(###\)\ ###\-####"/>
+    <numFmt numFmtId="164" formatCode="[&lt;=9999999]###\-####;\(###\)\ ###\-####"/>
+    <numFmt numFmtId="165" formatCode="0_);\(0\)"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="3" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="26"/>
+      <color theme="2" tint="-0.499984740745262"/>
+      <name val="Corbel"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="2" tint="-0.749961851863155"/>
+      <name val="Corbel"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="2" tint="-0.749961851863155"/>
+      <name val="Corbel"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -296,175 +366,19 @@
       <sz val="26"/>
       <color theme="3"/>
       <name val="Corbel"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="major"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="3" tint="-0.499984740745262"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="26"/>
-      <color theme="2" tint="-0.499984740745262"/>
-      <name val="Corbel"/>
-      <charset val="134"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
-      <color theme="2" tint="-0.749961851863155"/>
-      <name val="Corbel"/>
-      <charset val="134"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
-      <color theme="4"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="2" tint="-0.749961851863155"/>
-      <name val="Corbel"/>
-      <charset val="134"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -479,7 +393,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.0499893185216834"/>
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -489,187 +403,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="8">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="3" tint="-0.24994659260841701"/>
+      </top>
+      <bottom style="double">
+        <color theme="3" tint="-0.24994659260841701"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -692,422 +443,374 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="3" tint="-0.249946592608417"/>
-      </top>
-      <bottom style="double">
-        <color theme="3" tint="-0.249946592608417"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="56">
+  <cellStyleXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFill="0" applyBorder="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyFill="0" applyBorder="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="7" fontId="6" fillId="0" borderId="0" applyFill="0" applyBorder="0">
+    <xf numFmtId="7" fontId="4" fillId="2" borderId="0" applyFill="0" applyBorder="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="7" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="7" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0">
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyBorder="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFill="0" applyBorder="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="58" fontId="6" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyBorder="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="10">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="17">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="8">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="54">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="11">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="55">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="6">
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="12">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="16">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="7" fontId="6" fillId="2" borderId="1" xfId="2" applyFill="1" applyBorder="1">
+    <xf numFmtId="7" fontId="4" fillId="2" borderId="2" xfId="8" applyBorder="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="13">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="58" fontId="6" fillId="2" borderId="1" xfId="50" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="14">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="16">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="15">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="3" borderId="1" xfId="52" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="16" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="9" fillId="3" borderId="1" xfId="6" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="16" applyBorder="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="51">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="53" applyFont="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="49" applyFont="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="7" fontId="0" fillId="0" borderId="0" xfId="5" applyFont="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="7" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="5">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="2" borderId="2" xfId="12" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="18">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="7" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="15" applyFont="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="14" applyFont="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="7" fontId="0" fillId="0" borderId="0" xfId="9" applyFont="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="18">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="5">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="2">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="3">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="10">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="2" xfId="13" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="10" applyBorder="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" xfId="19" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="56">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
-    <cellStyle name="Date" xfId="49"/>
-    <cellStyle name="Inventory Date" xfId="50"/>
-    <cellStyle name="Item table heading" xfId="51"/>
-    <cellStyle name="Phone" xfId="52"/>
-    <cellStyle name="Seriel Number" xfId="53"/>
-    <cellStyle name="Title 2" xfId="54"/>
-    <cellStyle name="z Hidden Text" xfId="55"/>
+  <cellStyles count="20">
+    <cellStyle name="Comma" xfId="7" builtinId="3" customBuiltin="1"/>
+    <cellStyle name="Currency" xfId="8" builtinId="4" customBuiltin="1"/>
+    <cellStyle name="Currency [0]" xfId="9" builtinId="7" customBuiltin="1"/>
+    <cellStyle name="Date" xfId="14" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Heading 1" xfId="1" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="2" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="3" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="6" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Hyperlink" xfId="19" builtinId="8"/>
+    <cellStyle name="Input" xfId="10" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Inventory Date" xfId="12" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="Item table heading" xfId="17" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
+    <cellStyle name="Note" xfId="16" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Phone" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="Seriel Number" xfId="15" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
+    <cellStyle name="Title" xfId="5" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Title 2" xfId="11" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="Total" xfId="4" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="z Hidden Text" xfId="18" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="15">
     <dxf>
       <font>
-        <b val="1"/>
+        <b val="0"/>
         <i val="0"/>
-        <color theme="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2" tint="-0.749961851863155"/>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="5" tint="0.799951170384838"/>
-          <bgColor theme="2" tint="-0.0999481185338908"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="5" tint="0.799920651875362"/>
-          <bgColor theme="0" tint="-0.0499893185216834"/>
-        </patternFill>
-      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
         <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b val="0"/>
         <i val="0"/>
-        <color auto="1"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2"/>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="2" tint="-0.749961851863155"/>
+      </font>
       <border>
+        <bottom style="thin">
+          <color theme="2" tint="-0.499984740745262"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <sz val="11"/>
+        <color theme="1"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top/>
@@ -1118,7 +821,61 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.749961851863155"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="5" tint="0.79995117038483843"/>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="5" tint="0.79992065187536243"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <i val="0"/>
         <color theme="0"/>
       </font>
@@ -1142,48 +899,20 @@
         <color theme="3" tint="-0.499984740745262"/>
       </font>
     </dxf>
-    <dxf>
-      <font>
-        <color theme="2" tint="-0.749961851863155"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="2" tint="-0.499984740745262"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <sz val="11"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="Home Inventory" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Home Inventory" pivot="0" count="7" xr9:uid="{3B838D7D-2B0F-4A50-935F-26C9ED2F29C8}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="lastColumn" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="1"/>
-      <tableStyleElement type="firstTotalCell" dxfId="0"/>
+    <tableStyle name="Home Inventory" pivot="0" count="7" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" dxfId="14"/>
+      <tableStyleElement type="headerRow" dxfId="13"/>
+      <tableStyleElement type="totalRow" dxfId="12"/>
+      <tableStyleElement type="lastColumn" dxfId="11"/>
+      <tableStyleElement type="firstRowStripe" dxfId="10"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="9"/>
+      <tableStyleElement type="firstTotalCell" dxfId="8"/>
     </tableStyle>
-    <tableStyle name="Home Inventory Slicer" pivot="0" table="0" count="10" xr9:uid="{4EFDB511-9FC6-4204-9106-C4188F396082}">
-      <tableStyleElement type="wholeTable" dxfId="8"/>
-      <tableStyleElement type="headerRow" dxfId="7"/>
+    <tableStyle name="Home Inventory Slicer" pivot="0" table="0" count="10" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
+      <tableStyleElement type="wholeTable" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -1263,7 +992,8 @@
           </font>
           <fill>
             <patternFill patternType="solid">
-              <bgColor theme="0" tint="-0.349986266670736"/>
+              <fgColor auto="1"/>
+              <bgColor theme="0" tint="-0.34998626667073579"/>
             </patternFill>
           </fill>
           <border>
@@ -1289,7 +1019,8 @@
           </font>
           <fill>
             <patternFill patternType="solid">
-              <bgColor theme="0" tint="-0.249946592608417"/>
+              <fgColor auto="1"/>
+              <bgColor theme="0" tint="-0.24994659260841701"/>
             </patternFill>
           </fill>
           <border>
@@ -1315,10 +1046,11 @@
           </font>
           <fill>
             <patternFill patternType="solid">
+              <fgColor auto="1"/>
               <bgColor theme="5"/>
             </patternFill>
           </fill>
-          <border>
+          <border diagonalUp="0" diagonalDown="0">
             <left/>
             <right/>
             <top/>
@@ -1333,6 +1065,7 @@
           </font>
           <fill>
             <patternFill patternType="solid">
+              <fgColor auto="1"/>
               <bgColor theme="5"/>
             </patternFill>
           </fill>
@@ -1359,7 +1092,8 @@
           </font>
           <fill>
             <patternFill patternType="solid">
-              <bgColor theme="0" tint="-0.14996795556505"/>
+              <fgColor auto="1"/>
+              <bgColor theme="0" tint="-0.14996795556505021"/>
             </patternFill>
           </fill>
           <border>
@@ -1385,10 +1119,11 @@
           </font>
           <fill>
             <patternFill patternType="solid">
-              <bgColor theme="5" tint="0.399945066682943"/>
+              <fgColor auto="1"/>
+              <bgColor theme="5" tint="0.39994506668294322"/>
             </patternFill>
           </fill>
-          <border>
+          <border diagonalUp="0" diagonalDown="0">
             <left/>
             <right/>
             <top/>
@@ -1403,7 +1138,8 @@
           </font>
           <fill>
             <patternFill patternType="solid">
-              <bgColor theme="0" tint="-0.14996795556505"/>
+              <fgColor auto="1"/>
+              <bgColor theme="0" tint="-0.14996795556505021"/>
             </patternFill>
           </fill>
           <border>
@@ -1428,7 +1164,10 @@
             <color theme="1"/>
           </font>
           <fill>
-            <patternFill patternType="none"/>
+            <patternFill patternType="none">
+              <fgColor auto="1"/>
+              <bgColor auto="1"/>
+            </patternFill>
           </fill>
           <border>
             <left style="thin">
@@ -1465,12 +1204,15 @@
         </x14:slicerStyle>
       </x14:slicerStyles>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -1486,15 +1228,21 @@
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="19" name="Envelope icon group" descr="Envelope"/>
+        <xdr:cNvPr id="19" name="Envelope icon group" descr="Envelope">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000013000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGrpSpPr>
           <a:grpSpLocks noChangeAspect="1"/>
         </xdr:cNvGrpSpPr>
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="371475" y="1742440"/>
-          <a:ext cx="311150" cy="265430"/>
+          <a:off x="371481" y="1743074"/>
+          <a:ext cx="311230" cy="264883"/>
           <a:chOff x="1847850" y="4562475"/>
           <a:chExt cx="447675" cy="381000"/>
         </a:xfrm>
@@ -1504,12 +1252,20 @@
           </a:schemeClr>
         </a:solidFill>
       </xdr:grpSpPr>
-      <xdr:sp>
+      <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
-          <xdr:cNvPr id="20" name="Freeform 16"/>
-          <xdr:cNvSpPr/>
+          <xdr:cNvPr id="20" name="Freeform 16">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000014000000}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr>
+            <a:spLocks/>
+          </xdr:cNvSpPr>
         </xdr:nvSpPr>
-        <xdr:spPr>
+        <xdr:spPr bwMode="auto">
           <a:xfrm>
             <a:off x="1847850" y="4695825"/>
             <a:ext cx="447675" cy="247650"/>
@@ -2013,15 +1769,25 @@
             <a:noFill/>
             <a:prstDash val="solid"/>
             <a:round/>
+            <a:headEnd/>
+            <a:tailEnd/>
           </a:ln>
         </xdr:spPr>
       </xdr:sp>
-      <xdr:sp>
+      <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
-          <xdr:cNvPr id="21" name="Freeform 17"/>
-          <xdr:cNvSpPr/>
+          <xdr:cNvPr id="21" name="Freeform 17">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000015000000}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr>
+            <a:spLocks/>
+          </xdr:cNvSpPr>
         </xdr:nvSpPr>
-        <xdr:spPr>
+        <xdr:spPr bwMode="auto">
           <a:xfrm>
             <a:off x="1866900" y="4562475"/>
             <a:ext cx="409575" cy="209550"/>
@@ -2317,6 +2083,8 @@
             <a:noFill/>
             <a:prstDash val="solid"/>
             <a:round/>
+            <a:headEnd/>
+            <a:tailEnd/>
           </a:ln>
         </xdr:spPr>
       </xdr:sp>
@@ -2336,17 +2104,23 @@
       <xdr:row>3</xdr:row>
       <xdr:rowOff>155933</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="22" name="Person icon" descr="Person"/>
+        <xdr:cNvPr id="22" name="Person icon" descr="Person">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000016000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr>
           <a:spLocks noChangeAspect="1"/>
         </xdr:cNvSpPr>
       </xdr:nvSpPr>
-      <xdr:spPr>
+      <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="414020" y="1276350"/>
-          <a:ext cx="225425" cy="317500"/>
+          <a:off x="414524" y="1628775"/>
+          <a:ext cx="225144" cy="317858"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -2770,6 +2544,8 @@
           <a:noFill/>
           <a:prstDash val="solid"/>
           <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
         </a:ln>
       </xdr:spPr>
     </xdr:sp>
@@ -2790,15 +2566,21 @@
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="23" name="Telephone icon group" descr="Telephone"/>
+        <xdr:cNvPr id="23" name="Telephone icon group" descr="Telephone">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000017000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGrpSpPr>
           <a:grpSpLocks noChangeAspect="1"/>
         </xdr:cNvGrpSpPr>
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="377825" y="2238375"/>
-          <a:ext cx="297815" cy="244475"/>
+          <a:off x="378098" y="2238375"/>
+          <a:ext cx="297996" cy="245021"/>
           <a:chOff x="1857375" y="5410200"/>
           <a:chExt cx="428625" cy="352425"/>
         </a:xfrm>
@@ -2808,12 +2590,20 @@
           </a:schemeClr>
         </a:solidFill>
       </xdr:grpSpPr>
-      <xdr:sp>
+      <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
-          <xdr:cNvPr id="24" name="Freeform 20"/>
-          <xdr:cNvSpPr/>
+          <xdr:cNvPr id="24" name="Freeform 20">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000018000000}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr>
+            <a:spLocks/>
+          </xdr:cNvSpPr>
         </xdr:nvSpPr>
-        <xdr:spPr>
+        <xdr:spPr bwMode="auto">
           <a:xfrm>
             <a:off x="2190750" y="5486400"/>
             <a:ext cx="95250" cy="38100"/>
@@ -2973,15 +2763,25 @@
             <a:noFill/>
             <a:prstDash val="solid"/>
             <a:round/>
+            <a:headEnd/>
+            <a:tailEnd/>
           </a:ln>
         </xdr:spPr>
       </xdr:sp>
-      <xdr:sp>
+      <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
-          <xdr:cNvPr id="25" name="Freeform 21"/>
-          <xdr:cNvSpPr/>
+          <xdr:cNvPr id="25" name="Freeform 21">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000019000000}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr>
+            <a:spLocks/>
+          </xdr:cNvSpPr>
         </xdr:nvSpPr>
-        <xdr:spPr>
+        <xdr:spPr bwMode="auto">
           <a:xfrm>
             <a:off x="1866900" y="5486400"/>
             <a:ext cx="85725" cy="38100"/>
@@ -3141,17 +2941,25 @@
             <a:noFill/>
             <a:prstDash val="solid"/>
             <a:round/>
+            <a:headEnd/>
+            <a:tailEnd/>
           </a:ln>
         </xdr:spPr>
       </xdr:sp>
-      <xdr:sp>
+      <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
-          <xdr:cNvPr id="26" name="Freeform 22"/>
+          <xdr:cNvPr id="26" name="Freeform 22">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001A000000}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
           <xdr:cNvSpPr>
             <a:spLocks noEditPoints="1"/>
           </xdr:cNvSpPr>
         </xdr:nvSpPr>
-        <xdr:spPr>
+        <xdr:spPr bwMode="auto">
           <a:xfrm>
             <a:off x="1857375" y="5410200"/>
             <a:ext cx="428625" cy="352425"/>
@@ -4348,6 +4156,8 @@
             <a:noFill/>
             <a:prstDash val="solid"/>
             <a:round/>
+            <a:headEnd/>
+            <a:tailEnd/>
           </a:ln>
         </xdr:spPr>
       </xdr:sp>
@@ -4367,17 +4177,23 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>546170</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="29" name="House icon" descr="House"/>
+        <xdr:cNvPr id="29" name="House icon" descr="House">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001D000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr>
           <a:spLocks noChangeAspect="1" noEditPoints="1"/>
         </xdr:cNvSpPr>
       </xdr:nvSpPr>
-      <xdr:spPr>
+      <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="14253845" y="200025"/>
-          <a:ext cx="383540" cy="346075"/>
+          <a:off x="13873163" y="200031"/>
+          <a:ext cx="383760" cy="346139"/>
         </a:xfrm>
         <a:custGeom>
           <a:avLst/>
@@ -4965,6 +4781,8 @@
           <a:noFill/>
           <a:prstDash val="solid"/>
           <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
         </a:ln>
       </xdr:spPr>
     </xdr:sp>
@@ -4983,11 +4801,17 @@
       <xdr:row>8</xdr:row>
       <xdr:rowOff>847725</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer" Requires="sle15">
-        <xdr:graphicFrame>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+      <mc:Choice Requires="sle15">
+        <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="3" name="Room/&#10;area" descr="Room/Area slicer to filter items by Room/Area"/>
+            <xdr:cNvPr id="3" name="Room/&#10;area" descr="Room/Area slicer to filter items by Room/Area">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvGraphicFramePr/>
           </xdr:nvGraphicFramePr>
           <xdr:xfrm>
@@ -5011,7 +4835,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="212725" y="2638425"/>
+              <a:off x="212725" y="2628900"/>
               <a:ext cx="12131675" cy="790575"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -5031,9 +4855,9 @@
             <a:lstStyle/>
             <a:p>
               <a:r>
-                <a:rPr sz="1100"/>
-                <a:t>此形状表示切片器。
-当前版本不支持切片器，请升级到最新版的WPS。</a:t>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This shape represents a table slicer. Table slicers are supported in Excel or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2007 or earlier, the slicer can't be used.</a:t>
               </a:r>
             </a:p>
           </xdr:txBody>
@@ -5046,7 +4870,7 @@
 </file>
 
 <file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
-<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x" name="Slicer_Room__area" sourceName="Room/area">
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Room__area" xr10:uid="{00000000-0013-0000-FFFF-FFFF01000000}" sourceName="Room/area">
   <extLst>
     <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{2F2917AC-EB37-4324-AD4E-5DD8C200BD13}">
       <x15:tableSlicerCache tableId="1" column="3"/>
@@ -5056,45 +4880,55 @@
 </file>
 
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
-<slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <slicer name="Room/&#10;area" cache="Slicer_Room__area" caption="To filter your inventory list, select a room below. Hold Ctrl to select multiple rooms." columnCount="6" rowHeight="193675"/>
+<slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
+  <slicer name="Room/_x000a_area" xr10:uid="{00000000-0014-0000-FFFF-FFFF01000000}" cache="Slicer_Room__area" caption="To filter your inventory list, select a room below. Hold Ctrl to select multiple rooms." columnCount="6" rowHeight="193675"/>
 </slicers>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Inventory" displayName="Inventory" ref="B10:L16" totalsRowCount="1">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="B10:L15" etc:filterBottomFollowUsedRange="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Inventory" displayName="Inventory" ref="B10:L16" totalsRowCount="1">
+  <autoFilter ref="B10:L15" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="11">
-    <tableColumn id="21" name="Item #" totalsRowLabel="TOTALS">
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Item #" totalsRowLabel="TOTALS" dataCellStyle="Comma">
       <calculatedColumnFormula>ROW($A1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" name="Room/area" totalsRowFunction="custom">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Room/area" totalsRowFunction="custom" totalsRowDxfId="5">
       <totalsRowFormula>"INVENTORY ITEMS: "&amp;SUBTOTAL(103,Inventory[Room/area])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" name="Item/description"/>
-    <tableColumn id="5" name="Make/model"/>
-    <tableColumn id="6" name="Serial number/&#10;ID number"/>
-    <tableColumn id="7" name="Date&#10;purchased"/>
-    <tableColumn id="8" name="Where purchased"/>
-    <tableColumn id="9" name="Purchase&#10; price" totalsRowFunction="sum"/>
-    <tableColumn id="10" name="Estimated&#10;current value" totalsRowFunction="sum"/>
-    <tableColumn id="13" name="Notes"/>
-    <tableColumn id="14" name="Photo?"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Item/description" totalsRowDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Make/model" totalsRowDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Serial number/_x000a_ID number" dataCellStyle="Seriel Number"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Date_x000a_purchased" dataCellStyle="Date"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Where purchased" totalsRowDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Purchase_x000a_ price" totalsRowFunction="sum" dataCellStyle="Currency [0]"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Estimated_x000a_current value" totalsRowFunction="sum" dataCellStyle="Currency [0]"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Notes" totalsRowDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Photo?" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="Home Inventory" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{504A1905-F514-4f6f-8877-14C23A59335A}">
+      <x14:table altTextSummary="List of household inventory items such as, Item # (calculated field), Room/area, item information, Purchase information, Estimated Current Value, Notes, and Photo (Yes/No field)"/>
+    </ext>
+  </extLst>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoomLookup" displayName="RoomLookup" ref="B3:B15" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="B3:B15" etc:filterBottomFollowUsedRange="0"/>
-  <sortState ref="B3:B15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="RoomLookup" displayName="RoomLookup" ref="B3:B15" totalsRowShown="0">
+  <autoFilter ref="B3:B15" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:B15">
     <sortCondition ref="B3:B15"/>
   </sortState>
   <tableColumns count="1">
-    <tableColumn id="1" name="Room/Area"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Room/Area"/>
   </tableColumns>
   <tableStyleInfo name="Home Inventory" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{504A1905-F514-4f6f-8877-14C23A59335A}">
+      <x14:table altTextSummary="A table containing rooms or areas of a home"/>
+    </ext>
+  </extLst>
 </table>
 </file>
 
@@ -5233,51 +5067,74 @@
           <a:schemeClr val="phClr"/>
         </a:solidFill>
         <a:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+            <a:duotone>
+              <a:schemeClr val="phClr">
+                <a:shade val="90000"/>
+                <a:satMod val="140000"/>
+              </a:schemeClr>
+              <a:schemeClr val="phClr">
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:duotone>
+          </a:blip>
           <a:tile tx="0" ty="0" sx="100000" sy="100000" flip="none" algn="tl"/>
         </a:blipFill>
         <a:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+            <a:duotone>
+              <a:schemeClr val="phClr">
+                <a:shade val="90000"/>
+                <a:satMod val="140000"/>
+              </a:schemeClr>
+              <a:schemeClr val="phClr">
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:duotone>
+          </a:blip>
           <a:tile tx="0" ty="0" sx="100000" sy="100000" flip="none" algn="tl"/>
         </a:blipFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
-    <pageSetUpPr fitToPage="1" autoPageBreaks="0"/>
+    <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:L16"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.71428571428571" style="4" customWidth="1"/>
-    <col min="2" max="2" width="11.7142857142857" style="4" customWidth="1"/>
-    <col min="3" max="3" width="24.7142857142857" style="4" customWidth="1"/>
-    <col min="4" max="4" width="27.4285714285714" style="4" customWidth="1"/>
-    <col min="5" max="5" width="24.7142857142857" style="4" customWidth="1"/>
-    <col min="6" max="6" width="18.5714285714286" style="4" customWidth="1"/>
-    <col min="7" max="7" width="15.7142857142857" style="4" customWidth="1"/>
-    <col min="8" max="8" width="24.7142857142857" style="4" customWidth="1"/>
-    <col min="9" max="10" width="18.5714285714286" style="4" customWidth="1"/>
-    <col min="11" max="11" width="24.7142857142857" style="4" customWidth="1"/>
-    <col min="12" max="12" width="11.7142857142857" customWidth="1"/>
-    <col min="13" max="13" width="2.71428571428571" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="27.42578125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="18.5703125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="24.7109375" style="2" customWidth="1"/>
+    <col min="9" max="10" width="18.5703125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="24.7109375" style="2" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="13" width="2.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="65.25" customHeight="1" spans="1:12">
+    <row r="1" spans="1:12" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1"/>
+        <v>64</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="19"/>
       <c r="D1" s="5" t="s">
-        <v>2</v>
+        <v>53</v>
       </c>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
@@ -5286,165 +5143,165 @@
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
       <c r="K1" s="3"/>
-      <c r="L1" s="6" t="s">
-        <v>3</v>
+      <c r="L1" s="13" t="s">
+        <v>55</v>
       </c>
     </row>
-    <row r="2" customHeight="1" spans="1:12">
+    <row r="2" spans="1:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
-      <c r="B2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="8">
+      <c r="B2" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="9">
         <f>SUM(Inventory[[#Totals],[Estimated
 current value]])</f>
         <v>4040</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="9"/>
-      <c r="I2" s="10">
+      <c r="F2" s="8"/>
+      <c r="G2" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="H2" s="21"/>
+      <c r="I2" s="12">
         <f ca="1">TODAY()-35</f>
-        <v>46222</v>
-      </c>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
+        <v>45743</v>
+      </c>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
     </row>
-    <row r="3" ht="18" customHeight="1" spans="1:12">
+    <row r="3" spans="1:12" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
-      <c r="B3" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
+      <c r="B3" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
       <c r="G3" s="3"/>
-      <c r="H3" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
+      <c r="H3" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
       <c r="L3" s="3"/>
     </row>
-    <row r="4" ht="18" customHeight="1" spans="1:12">
+    <row r="4" spans="1:12" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
       <c r="G4" s="3"/>
-      <c r="H4" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="I4" s="14">
+      <c r="H4" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="24">
         <v>866699666</v>
       </c>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
       <c r="L4" s="3"/>
     </row>
-    <row r="5" ht="18" customHeight="1" spans="1:12">
+    <row r="5" spans="1:12" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
-      <c r="B5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
+      <c r="B5" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
       <c r="G5" s="3"/>
-      <c r="H5" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="I5" s="15">
-        <v>321000000000000</v>
-      </c>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
+      <c r="H5" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="23">
+        <v>321789546489000</v>
+      </c>
+      <c r="J5" s="23"/>
+      <c r="K5" s="23"/>
       <c r="L5" s="3"/>
     </row>
-    <row r="6" ht="18" customHeight="1" spans="1:12">
+    <row r="6" spans="1:12" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
       <c r="G6" s="3"/>
-      <c r="H6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="I6" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="L6" s="16"/>
+      <c r="H6" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="4"/>
     </row>
-    <row r="7" ht="18" customHeight="1" spans="1:12">
+    <row r="7" spans="1:12" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
-      <c r="B7" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
+      <c r="B7" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
       <c r="G7" s="3"/>
-      <c r="H7" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="I7" s="14">
+      <c r="H7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="24">
         <v>869909986</v>
       </c>
-      <c r="J7" s="14"/>
-      <c r="K7" s="14"/>
+      <c r="J7" s="24"/>
+      <c r="K7" s="24"/>
       <c r="L7" s="3"/>
     </row>
-    <row r="8" ht="18" customHeight="1" spans="1:12">
+    <row r="8" spans="1:12" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
       <c r="G8" s="3"/>
-      <c r="H8" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I8" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
+      <c r="H8" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="J8" s="25"/>
+      <c r="K8" s="25"/>
       <c r="L8" s="3"/>
     </row>
-    <row r="9" ht="69" customHeight="1" spans="1:12">
+    <row r="9" spans="1:12" ht="69" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
-      <c r="B9" s="6" t="s">
-        <v>24</v>
+      <c r="B9" s="13" t="s">
+        <v>63</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -5457,220 +5314,220 @@
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
     </row>
-    <row r="10" customHeight="1" spans="1:12">
-      <c r="B10" s="19" t="s">
-        <v>25</v>
+    <row r="10" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>57</v>
       </c>
       <c r="E10" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" t="s">
+        <v>2</v>
+      </c>
+      <c r="G10" t="s">
         <v>28</v>
       </c>
-      <c r="F10" t="s">
+      <c r="H10" t="s">
+        <v>3</v>
+      </c>
+      <c r="I10" t="s">
+        <v>4</v>
+      </c>
+      <c r="J10" t="s">
         <v>29</v>
       </c>
-      <c r="G10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I10" t="s">
-        <v>32</v>
-      </c>
-      <c r="J10" t="s">
-        <v>33</v>
-      </c>
       <c r="K10" t="s">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>35</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="11" customHeight="1" spans="1:12">
-      <c r="B11" s="20">
+    <row r="11" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="14">
         <f>ROW($A1)</f>
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="G11" s="22">
+        <v>47</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="16">
         <f ca="1">TODAY()-120</f>
-        <v>46137</v>
+        <v>45658</v>
       </c>
       <c r="H11" t="s">
-        <v>40</v>
-      </c>
-      <c r="I11" s="23">
+        <v>16</v>
+      </c>
+      <c r="I11" s="17">
         <v>2000</v>
       </c>
-      <c r="J11" s="23">
+      <c r="J11" s="17">
         <v>2000</v>
       </c>
       <c r="K11"/>
       <c r="L11" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
     </row>
-    <row r="12" customHeight="1" spans="1:12">
-      <c r="B12" s="20">
+    <row r="12" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="14">
         <f t="shared" ref="B12:B15" si="0">ROW($A2)</f>
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>44</v>
-      </c>
-      <c r="F12" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="G12" s="22">
+        <v>48</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="16">
         <f ca="1">TODAY()-90</f>
-        <v>46167</v>
+        <v>45688</v>
       </c>
       <c r="H12" t="s">
-        <v>46</v>
-      </c>
-      <c r="I12" s="23">
+        <v>31</v>
+      </c>
+      <c r="I12" s="17">
         <v>1500</v>
       </c>
-      <c r="J12" s="23">
+      <c r="J12" s="17">
         <v>1000</v>
       </c>
       <c r="K12"/>
       <c r="L12" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
     </row>
-    <row r="13" customHeight="1" spans="1:12">
+    <row r="13" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13"/>
-      <c r="B13" s="20">
+      <c r="B13" s="14">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="D13" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="E13" t="s">
         <v>49</v>
       </c>
-      <c r="F13" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="G13" s="22">
+      <c r="F13" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" s="16">
         <f ca="1">TODAY()-60</f>
-        <v>46197</v>
+        <v>45718</v>
       </c>
       <c r="H13" t="s">
-        <v>51</v>
-      </c>
-      <c r="I13" s="23">
+        <v>39</v>
+      </c>
+      <c r="I13" s="17">
         <v>560</v>
       </c>
-      <c r="J13" s="23">
+      <c r="J13" s="17">
         <v>550</v>
       </c>
       <c r="K13"/>
       <c r="L13" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
     </row>
-    <row r="14" customHeight="1" spans="1:12">
-      <c r="B14" s="20">
+    <row r="14" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="14">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="E14" t="s">
-        <v>54</v>
-      </c>
-      <c r="F14" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="G14" s="22">
+        <v>50</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="G14" s="16">
         <f ca="1">TODAY()-30</f>
-        <v>46227</v>
+        <v>45748</v>
       </c>
       <c r="H14" t="s">
-        <v>40</v>
-      </c>
-      <c r="I14" s="23">
+        <v>16</v>
+      </c>
+      <c r="I14" s="17">
         <v>240</v>
       </c>
-      <c r="J14" s="23">
+      <c r="J14" s="17">
         <v>200</v>
       </c>
       <c r="K14"/>
       <c r="L14" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
     </row>
-    <row r="15" customHeight="1" spans="1:12">
-      <c r="B15" s="20">
+    <row r="15" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="14">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="E15" t="s">
-        <v>58</v>
-      </c>
-      <c r="F15" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="G15" s="22">
+        <v>51</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="G15" s="16">
         <f ca="1">TODAY()</f>
-        <v>46257</v>
+        <v>45778</v>
       </c>
       <c r="H15" t="s">
-        <v>46</v>
-      </c>
-      <c r="I15" s="23">
+        <v>31</v>
+      </c>
+      <c r="I15" s="17">
         <v>300</v>
       </c>
-      <c r="J15" s="23">
+      <c r="J15" s="17">
         <v>290</v>
       </c>
       <c r="K15"/>
       <c r="L15" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
     </row>
-    <row r="16" customHeight="1" spans="1:12">
+    <row r="16" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="C16" s="3" t="str">
         <f>"INVENTORY ITEMS: "&amp;SUBTOTAL(103,Inventory[Room/area])</f>
@@ -5681,12 +5538,12 @@
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
-      <c r="I16" s="24">
+      <c r="I16" s="10">
         <f>SUBTOTAL(109,Inventory[Purchase
  price])</f>
         <v>4600</v>
       </c>
-      <c r="J16" s="24">
+      <c r="J16" s="10">
         <f>SUBTOTAL(109,Inventory[Estimated
 current value])</f>
         <v>4040</v>
@@ -5695,26 +5552,28 @@
       <c r="L16" s="3"/>
     </row>
   </sheetData>
+  <dataConsolidate/>
   <mergeCells count="18">
+    <mergeCell ref="I6:K6"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="D7:F8"/>
+    <mergeCell ref="D5:F6"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="B7:B8"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="G2:H2"/>
-    <mergeCell ref="I3:K3"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="I6:K6"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="C5:C6"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="D7:F8"/>
-    <mergeCell ref="D5:F6"/>
+    <mergeCell ref="B3:B4"/>
   </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="J11:J15">
     <cfRule type="dataBar" priority="1">
       <dataBar>
@@ -5724,70 +5583,70 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{99af1854-487a-4040-9322-737d525e1428}</x14:id>
+          <x14:id>{DD2554B5-7481-4F06-9B0C-4C198BA00901}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="31">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Create a Home inventory in this workbook. Enter owner, insurance, and inventory details in this worksheet. Total estimated value of all inventory items is automatically calculated" sqref="A1"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Title of this worksheet is in cells B1 through D1" sqref="B1:C1"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Total Estimated Value of All Items is automatically calculated in cell at right. Enter Inventory Date in cell I2" sqref="B2:D2"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Total Estimated Value of All Items is automatically calculated in this cell. Enter Inventory Date in cell I2" sqref="E2"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Inventory Date in cell at right" sqref="G2:H2"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Inventory Date in this cell" sqref="I2"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance company name in cell at right" sqref="H3"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance company phone number in cell at right" sqref="H4"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance company policy number in cell at right" sqref="H5"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance agent name in cell at right" sqref="H6"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance agent phone number in cell at right" sqref="H7"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance agent address in cell at right" sqref="H8"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance agent address in this cell, and inventory details in table starting in cell B10. Use slicer in cell B9 to filter items by Room/Area" sqref="I8:K8"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Item number in this column under this heading. Use heading filters to find specific entries" sqref="B10"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Select Room/area in this column under this heading. Enter new Room/Area in Room Lookup worksheet. Press ALT+DOWN ARROW for options, then DOWN ARROW and ENTER to make selection" sqref="C10"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Item/description in this column under this heading" sqref="D10"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Make/model in this column under this heading" sqref="E10"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Serial number/ID number in this column under this heading" sqref="F10"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Date purchased in this column under this heading" sqref="G10"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Where purchased in this column under this heading" sqref="H10"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Purchase price in this column under this heading" sqref="I10"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Estimated current value in this column under this heading. Data bar showing Estimated current value is automatically updated in each row" sqref="J10"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Notes in this column under this heading" sqref="K10"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Select &quot;Yes&quot; if Photo of the item exists, otherwise &quot;No&quot; in this column under this heading. Press ALT+DOWN ARROW for options, then DOWN ARROW and ENTER to make selection" sqref="L10"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter personal details in cells C3 through E8 and Insurance information in cells H3 through K8" sqref="B3:B4"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Data" error="Please select an entry from the list. To add or change items, use the Room/Area table on the Room Lookup worksheet. " sqref="B11:B15"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter owner Name in cell at right" sqref="C3:C4"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter owner Address in cell at right" sqref="C5:C6"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter owner Phone number in cell at right" sqref="C7:C8"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Select Room/area from the list. Enter new Room/Area in Room Lookup worksheet. Select CANCEL, then press ALT+DOWN ARROW for options, then DOWN ARROW and ENTER to make selection" sqref="C11:C15" errorStyle="warning">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Title of this worksheet is in cells B1 through D1" sqref="B1:C1" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Total Estimated Value of All Items is automatically calculated in cell at right. Enter Inventory Date in cell I2" sqref="B2:D2" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Total Estimated Value of All Items is automatically calculated in this cell. Enter Inventory Date in cell I2" sqref="E2" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Inventory Date in cell at right" sqref="G2:H2" xr:uid="{00000000-0002-0000-0000-000003000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Inventory Date in this cell" sqref="I2" xr:uid="{00000000-0002-0000-0000-000004000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter owner Name in cell at right" sqref="C3:C4" xr:uid="{00000000-0002-0000-0000-000005000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter owner Address in cell at right" sqref="C5:C6" xr:uid="{00000000-0002-0000-0000-000006000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter owner Phone number in cell at right" sqref="C7:C8" xr:uid="{00000000-0002-0000-0000-000007000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance company name in cell at right" sqref="H3" xr:uid="{00000000-0002-0000-0000-000008000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance company phone number in cell at right" sqref="H4" xr:uid="{00000000-0002-0000-0000-000009000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance company policy number in cell at right" sqref="H5" xr:uid="{00000000-0002-0000-0000-00000A000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance agent name in cell at right" sqref="H6" xr:uid="{00000000-0002-0000-0000-00000B000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance agent phone number in cell at right" sqref="H7" xr:uid="{00000000-0002-0000-0000-00000C000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance agent address in cell at right" sqref="H8" xr:uid="{00000000-0002-0000-0000-00000D000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Insurance agent address in this cell, and inventory details in table starting in cell B10. Use slicer in cell B9 to filter items by Room/Area" sqref="I8:K8" xr:uid="{00000000-0002-0000-0000-00000E000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Create a Home inventory in this workbook. Enter owner, insurance, and inventory details in this worksheet. Total estimated value of all inventory items is automatically calculated" sqref="A1" xr:uid="{00000000-0002-0000-0000-00000F000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Item number in this column under this heading. Use heading filters to find specific entries" sqref="B10" xr:uid="{00000000-0002-0000-0000-000010000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Item/description in this column under this heading" sqref="D10" xr:uid="{00000000-0002-0000-0000-000011000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Select Room/area in this column under this heading. Enter new Room/Area in Room Lookup worksheet. Press ALT+DOWN ARROW for options, then DOWN ARROW and ENTER to make selection" sqref="C10" xr:uid="{00000000-0002-0000-0000-000012000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Make/model in this column under this heading" sqref="E10" xr:uid="{00000000-0002-0000-0000-000013000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Serial number/ID number in this column under this heading" sqref="F10" xr:uid="{00000000-0002-0000-0000-000014000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Date purchased in this column under this heading" sqref="G10" xr:uid="{00000000-0002-0000-0000-000015000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Where purchased in this column under this heading" sqref="H10" xr:uid="{00000000-0002-0000-0000-000016000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Purchase price in this column under this heading" sqref="I10" xr:uid="{00000000-0002-0000-0000-000017000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Estimated current value in this column under this heading. Data bar showing Estimated current value is automatically updated in each row" sqref="J10" xr:uid="{00000000-0002-0000-0000-000018000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter Notes in this column under this heading" sqref="K10" xr:uid="{00000000-0002-0000-0000-000019000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Select &quot;Yes&quot; if Photo of the item exists, otherwise &quot;No&quot; in this column under this heading. Press ALT+DOWN ARROW for options, then DOWN ARROW and ENTER to make selection" sqref="L10" xr:uid="{00000000-0002-0000-0000-00001A000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter personal details in cells C3 through E8 and Insurance information in cells H3 through K8" sqref="B3:B4" xr:uid="{00000000-0002-0000-0000-00001B000000}"/>
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Select Yes or No from the list to indicate whether a photo of the item exists. Select CANCEL, then press ALT+DOWN ARROW for options, then DOWN ARROW and ENTER to make selection" sqref="L11:L15" xr:uid="{00000000-0002-0000-0000-00001C000000}">
+      <formula1>"Yes, No"</formula1>
+    </dataValidation>
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Select Room/area from the list. Enter new Room/Area in Room Lookup worksheet. Select CANCEL, then press ALT+DOWN ARROW for options, then DOWN ARROW and ENTER to make selection" sqref="C11:C15" xr:uid="{00000000-0002-0000-0000-00001D000000}">
       <formula1>RoomList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Select Yes or No from the list to indicate whether a photo of the item exists. Select CANCEL, then press ALT+DOWN ARROW for options, then DOWN ARROW and ENTER to make selection" sqref="L11:L15" errorStyle="warning">
-      <formula1>"Yes, No"</formula1>
-    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Data" error="Please select an entry from the list. To add or change items, use the Room/Area table on the Room Lookup worksheet. " sqref="B11:B15" xr:uid="{00000000-0002-0000-0000-00001E000000}"/>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="D7" r:id="rId4" display="roy.wang@aspose.com"/>
+    <hyperlink ref="D7" r:id="rId1" xr:uid="{F6F0B196-1857-4923-B3E1-3F9793F92971}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" scale="59" fitToHeight="0" orientation="landscape"/>
+  <pageSetup scale="59" fitToHeight="0" orientation="landscape" r:id="rId2"/>
   <headerFooter differentFirst="1">
-    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <ignoredErrors>
     <ignoredError sqref="F14" numberStoredAsText="1"/>
     <ignoredError sqref="B11:B15" emptyCellReference="1"/>
   </ignoredErrors>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{99af1854-487a-4040-9322-737d525e1428}">
+          <x14:cfRule type="dataBar" id="{DD2554B5-7481-4F06-9B0C-4C198BA00901}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -5799,9 +5658,9 @@
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
-      <x14:slicerList>
-        <x14:slicer r:id="rId3"/>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{3A4CF648-6AED-40f4-86FF-DC5316D8AED3}">
+      <x14:slicerList xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
+        <x14:slicer r:id="rId5"/>
       </x14:slicerList>
     </ext>
   </extLst>
@@ -5809,108 +5668,115 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="5"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:B15"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1" outlineLevelCol="1"/>
+  <sheetFormatPr defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.71428571428571" customWidth="1"/>
-    <col min="2" max="2" width="50.5714285714286" customWidth="1"/>
-    <col min="3" max="3" width="2.71428571428571" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" customWidth="1"/>
+    <col min="2" max="2" width="50.5703125" customWidth="1"/>
+    <col min="3" max="3" width="2.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35.25" customHeight="1" spans="2:2">
-      <c r="B1" s="1" t="s">
-        <v>61</v>
+    <row r="1" spans="2:2" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="11" t="s">
+        <v>59</v>
       </c>
     </row>
-    <row r="2" ht="50.25" customHeight="1" spans="2:2">
-      <c r="B2" s="2" t="s">
-        <v>62</v>
+    <row r="2" spans="2:2" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="7" t="s">
+        <v>54</v>
       </c>
     </row>
-    <row r="3" customHeight="1" spans="2:2">
+    <row r="3" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>63</v>
+        <v>15</v>
       </c>
     </row>
-    <row r="4" customHeight="1" spans="2:2">
+    <row r="4" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
     </row>
-    <row r="5" customHeight="1" spans="2:2">
+    <row r="5" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
-        <v>65</v>
+        <v>9</v>
       </c>
     </row>
-    <row r="6" customHeight="1" spans="2:2">
+    <row r="6" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
-        <v>66</v>
+        <v>10</v>
       </c>
     </row>
-    <row r="7" customHeight="1" spans="2:2">
+    <row r="7" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
-        <v>67</v>
+        <v>11</v>
       </c>
     </row>
-    <row r="8" customHeight="1" spans="2:2">
+    <row r="8" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
-        <v>68</v>
+        <v>46</v>
       </c>
     </row>
-    <row r="9" customHeight="1" spans="2:2">
+    <row r="9" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
     </row>
-    <row r="10" customHeight="1" spans="2:2">
+    <row r="10" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
-        <v>56</v>
+        <v>13</v>
       </c>
     </row>
-    <row r="11" customHeight="1" spans="2:2">
+    <row r="11" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
-        <v>69</v>
+        <v>12</v>
       </c>
     </row>
-    <row r="12" customHeight="1" spans="2:2">
+    <row r="12" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
-        <v>42</v>
+        <v>14</v>
       </c>
     </row>
-    <row r="13" customHeight="1" spans="2:2">
+    <row r="13" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
-        <v>70</v>
+        <v>7</v>
       </c>
     </row>
-    <row r="14" customHeight="1" spans="2:2">
+    <row r="14" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
-        <v>36</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="15" customHeight="1" spans="2:2">
+    <row r="15" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
-        <v>71</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
+  <dataConsolidate/>
   <dataValidations count="3">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Create a list of rooms or areas in this worksheet. Customize Room/Area selection in Inventory table by inserting or modifying Room/Area in Room Lookup table in this worksheet" sqref="A1"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Title of this worksheet is in this cell" sqref="B1"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Room or Areas are in this column under this heading" sqref="B3"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Create a list of rooms or areas in this worksheet. Customize Room/Area selection in Inventory table by inserting or modifying Room/Area in Room Lookup table in this worksheet" sqref="A1" xr:uid="{00000000-0002-0000-0100-000000000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Title of this worksheet is in this cell" sqref="B1" xr:uid="{00000000-0002-0000-0100-000001000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Room or Areas are in this column under this heading" sqref="B3" xr:uid="{00000000-0002-0000-0100-000002000000}"/>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" fitToHeight="0" orientation="portrait"/>
+  <pageSetup fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter differentFirst="1">
-    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <oddFooter>Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{f42aa342-8706-4288-bd11-ebb85995028c}" enabled="1" method="Standard" siteId="{72f988bf-86f1-41af-91ab-2d7cd011db47}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>